<commit_message>
feat(backend): update master word and excel templates with all 6 question types
</commit_message>
<xml_diff>
--- a/apps/backend/src/modules/question-bank/templates/default-template-soal.xlsx
+++ b/apps/backend/src/modules/question-bank/templates/default-template-soal.xlsx
@@ -6,16 +6,15 @@
   <sheets>
     <sheet sheetId="1" name="📋 Panduan" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="✍️ Input Soal" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="💡 Contoh Soal" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="55">
-  <si>
-    <t>ASSESSIA BY ORIVASTRA - PETUNJUK TEMPLATE EXCEL</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="69">
+  <si>
+    <t>ASSESSIA BY ORIVASTRA - PETUNJUK TEMPLATE EXCEL MULTI-TIPE</t>
   </si>
   <si>
     <t/>
@@ -39,6 +38,15 @@
     <t>1, 2, 3...</t>
   </si>
   <si>
+    <t>Tipe Soal</t>
+  </si>
+  <si>
+    <t>PILIH DARI DROPDOWN MENU (PILIHAN GANDA, PG KOMPLEKS, BENAR SALAH, ISIAN SINGKAT, MENJODOHKAN, ESAI)</t>
+  </si>
+  <si>
+    <t>PILIHAN GANDA (Tersedia menu dropdown)</t>
+  </si>
+  <si>
     <t>Soal</t>
   </si>
   <si>
@@ -51,28 +59,28 @@
     <t>Opsi A s.d. E</t>
   </si>
   <si>
-    <t>Pilihan jawaban A sampai E</t>
-  </si>
-  <si>
-    <t>Jakarta (pada kolom Opsi A)</t>
+    <t>Pilihan jawaban A sampai E. Untuk Menjodohkan gunakan format: Pernyataan -&gt; Pasangan. Kosongkan untuk Benar/Salah, Isian, dan Esai.</t>
+  </si>
+  <si>
+    <t>Jakarta (Opsi A) atau Kartini -&gt; Jepara</t>
   </si>
   <si>
     <t>Kunci Jawaban</t>
   </si>
   <si>
-    <t>PILIH DARI DROPDOWN MENU (A, B, C, D, atau E)</t>
-  </si>
-  <si>
-    <t>A (Tersedia menu pilihan otomatis)</t>
+    <t>PG: A-E | PG Kompleks: A, B, D | Benar Salah: BENAR / SALAH | Isian: Kata kunci | Menjodohkan &amp; Esai: Kosongkan</t>
+  </si>
+  <si>
+    <t>B (PG) atau A, B, D (Kompleks)</t>
   </si>
   <si>
     <t>Pembahasan (Opsional)</t>
   </si>
   <si>
-    <t>Penjelasan rinci untuk evaluasi siswa</t>
-  </si>
-  <si>
-    <t>Jakarta merupakan pusat pemerintahan.</t>
+    <t>Penjelasan rinci untuk evaluasi dan rubrik siswa</t>
+  </si>
+  <si>
+    <t>Nusantara di Kalimantan Timur.</t>
   </si>
   <si>
     <t>Tingkat Kesulitan</t>
@@ -84,7 +92,7 @@
     <t>SEDANG (Default jika dikosongkan)</t>
   </si>
   <si>
-    <t>💡 TIPS: Buka lembar "✍️ Input Soal" di tab bawah untuk mulai mengisi soal. Gunakan menu dropdown pada kolom Kunci Jawaban agar terhindar dari salah ketik.</t>
+    <t>💡 TIPS: Buka lembar "✍️ Input Soal" di tab bawah untuk mulai mengisi soal. Kolom Tipe Soal memudahkan Assessia mengenali format soal secara otomatis tanpa resiko salah tafsir.</t>
   </si>
   <si>
     <t>Opsi A</t>
@@ -102,82 +110,115 @@
     <t>Opsi E</t>
   </si>
   <si>
+    <t>PILIHAN GANDA</t>
+  </si>
+  <si>
     <t>Perangkat lunak berikut ini yang berfungsi sebagai sistem operasi pada komputer adalah...</t>
   </si>
   <si>
     <t>Microsoft Word</t>
   </si>
   <si>
-    <t>Microsoft Windows</t>
+    <t>Linux Ubuntu</t>
+  </si>
+  <si>
+    <t>Adobe Photoshop</t>
   </si>
   <si>
     <t>Google Chrome</t>
   </si>
   <si>
-    <t>Adobe Photoshop</t>
-  </si>
-  <si>
-    <t>Visual Studio Code</t>
+    <t>VLC Media Player</t>
   </si>
   <si>
     <t>B</t>
   </si>
   <si>
-    <t>Microsoft Windows merupakan sistem operasi yang mengelola perangkat lunak dan keras.</t>
+    <t>Linux Ubuntu merupakan sistem operasi komputer open-source berbasis kernel Linux.</t>
   </si>
   <si>
     <t>MUDAH</t>
   </si>
   <si>
-    <t>Jika diketahui persamaan kuadrat 2x² + 5x - 3 = 0, maka nilai diskriminan (D) adalah...</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>49</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
-    <t>-1</t>
-  </si>
-  <si>
-    <t>Rumus diskriminan D = b² - 4ac. Nilai D = (5)² - 4(2)(-3) = 25 + 24 = 49.</t>
+    <t>PG KOMPLEKS</t>
+  </si>
+  <si>
+    <t>Manakah dari bahasa pemrograman berikut yang dieksekusi secara interpreted?</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>JavaScript</t>
+  </si>
+  <si>
+    <t>C++</t>
+  </si>
+  <si>
+    <t>Ruby</t>
+  </si>
+  <si>
+    <t>A, B, D</t>
+  </si>
+  <si>
+    <t>Python, JavaScript, dan Ruby diinterpretasi oleh runtime engine.</t>
   </si>
   <si>
     <t>SEDANG</t>
   </si>
   <si>
-    <t>Microsoft Windows merupakan sistem operasi yang mengelola perangkat komputer.</t>
-  </si>
-  <si>
-    <t>Rumus D = b² - 4ac = (5)² - 4(2)(-3) = 25 + 24 = 49.</t>
-  </si>
-  <si>
-    <t>Organel sel yang berfungsi sebagai tempat respirasi seluler dan penghasil energi utama (ATP) adalah...</t>
-  </si>
-  <si>
-    <t>Ribosom</t>
-  </si>
-  <si>
-    <t>Mitokondria</t>
-  </si>
-  <si>
-    <t>Retikulum Endoplasma</t>
-  </si>
-  <si>
-    <t>Lisosom</t>
-  </si>
-  <si>
-    <t>Badan Golgi</t>
-  </si>
-  <si>
-    <t>Mitokondria merupakan the powerhouse of the cell penghasil ATP.</t>
+    <t>BENAR SALAH</t>
+  </si>
+  <si>
+    <t>Fotosintesis pada tumbuhan hijau menghasilkan oksigen dan senyawa glukosa.</t>
+  </si>
+  <si>
+    <t>BENAR</t>
+  </si>
+  <si>
+    <t>Reaksi fotosintesis menghasilkan C6H12O6 dan gas O2.</t>
+  </si>
+  <si>
+    <t>ISIAN SINGKAT</t>
+  </si>
+  <si>
+    <t>Bahasa resmi yang digunakan oleh penduduk negara Brazil adalah...</t>
+  </si>
+  <si>
+    <t>Portugis, portugis</t>
+  </si>
+  <si>
+    <t>Brazil merupakan satu-satunya negara berbahasa resmi Portugis di benua Amerika Selatan.</t>
+  </si>
+  <si>
+    <t>MENJODOHKAN</t>
+  </si>
+  <si>
+    <t>Jodohkanlah nama pahlawan nasional berikut dengan kota asalnya:</t>
+  </si>
+  <si>
+    <t>R.A. Kartini -&gt; Jepara</t>
+  </si>
+  <si>
+    <t>Pangeran Diponegoro -&gt; Yogyakarta</t>
+  </si>
+  <si>
+    <t>Cut Nyak Dien -&gt; Aceh</t>
+  </si>
+  <si>
+    <t>Kartini berasal dari Jepara, Diponegoro dari Yogyakarta, Cut Nyak Dien dari Aceh.</t>
+  </si>
+  <si>
+    <t>SULIT</t>
+  </si>
+  <si>
+    <t>ESAI</t>
+  </si>
+  <si>
+    <t>Jelaskan perbedaan mendasar antara siklus lisogenik dan litik pada replikasi virus!</t>
+  </si>
+  <si>
+    <t>Siklus litik melisiskan sel inang segera setelah replikasi, sedangkan siklus lisogenik menyisipkan materi genetik virus ke kromosom sel inang.</t>
   </si>
 </sst>
 </file>
@@ -216,7 +257,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -241,11 +282,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="1E293B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0F766E"/>
       </patternFill>
     </fill>
   </fills>
@@ -279,7 +315,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -301,9 +337,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -647,13 +680,13 @@
   <sheetPr>
     <tabColor rgb="2563EB"/>
   </sheetPr>
-  <dimension ref="A2:D13"/>
+  <dimension ref="A2:D14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="45" customWidth="1"/>
-    <col min="4" max="4" width="35" customWidth="1"/>
+    <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="4" max="4" width="38" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" ht="35" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
@@ -663,7 +696,7 @@
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="4" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -677,7 +710,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -691,7 +724,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -705,7 +738,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -719,7 +752,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -733,7 +766,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -747,7 +780,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -761,22 +794,36 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B12" s="4" t="s">
+    <row r="11" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
+      <c r="C11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B13" s="4"/>
+      <c r="B13" s="4" t="s">
+        <v>26</v>
+      </c>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B12:D13"/>
+    <mergeCell ref="B13:D14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -788,18 +835,19 @@
   <sheetPr>
     <tabColor rgb="10B981"/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="3" max="7" width="25" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="35" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="45" customWidth="1"/>
+    <col min="4" max="8" width="25" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="35" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" ht="32" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>5</v>
       </c>
@@ -807,22 +855,22 @@
         <v>8</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="I1" s="5" t="s">
         <v>17</v>
@@ -830,1035 +878,1031 @@
       <c r="J1" s="5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="H2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="I2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="J2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="K2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1</v>
+      </c>
+      <c r="I3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I4" t="s">
+        <v>53</v>
+      </c>
+      <c r="J4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K4" t="s">
         <v>41</v>
       </c>
-      <c r="F3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G3" t="s">
-        <v>43</v>
-      </c>
-      <c r="H3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3" t="s">
-        <v>44</v>
-      </c>
-      <c r="J3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="6">
-        <v>3</v>
-      </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="6"/>
-    </row>
-    <row r="5" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="6">
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="6"/>
-    </row>
-    <row r="6" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="6">
+      <c r="B5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I5" t="s">
+        <v>57</v>
+      </c>
+      <c r="J5" t="s">
+        <v>58</v>
+      </c>
+      <c r="K5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="6"/>
-    </row>
-    <row r="7" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="6">
+      <c r="B6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6" t="s">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>1</v>
+      </c>
+      <c r="J6" t="s">
+        <v>64</v>
+      </c>
+      <c r="K6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="6"/>
-    </row>
-    <row r="8" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>1</v>
+      </c>
+      <c r="J7" t="s">
+        <v>68</v>
+      </c>
+      <c r="K7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="6">
         <v>7</v>
       </c>
-      <c r="B8" s="7"/>
+      <c r="B8" s="6"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
       <c r="G8" s="7"/>
-      <c r="H8" s="6"/>
+      <c r="H8" s="7"/>
       <c r="I8" s="7"/>
-      <c r="J8" s="6"/>
-    </row>
-    <row r="9" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J8" s="7"/>
+      <c r="K8" s="6"/>
+    </row>
+    <row r="9" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="6">
         <v>8</v>
       </c>
-      <c r="B9" s="7"/>
+      <c r="B9" s="6"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
-      <c r="H9" s="6"/>
+      <c r="H9" s="7"/>
       <c r="I9" s="7"/>
-      <c r="J9" s="6"/>
-    </row>
-    <row r="10" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J9" s="7"/>
+      <c r="K9" s="6"/>
+    </row>
+    <row r="10" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="6">
         <v>9</v>
       </c>
-      <c r="B10" s="7"/>
+      <c r="B10" s="6"/>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
-      <c r="H10" s="6"/>
+      <c r="H10" s="7"/>
       <c r="I10" s="7"/>
-      <c r="J10" s="6"/>
-    </row>
-    <row r="11" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J10" s="7"/>
+      <c r="K10" s="6"/>
+    </row>
+    <row r="11" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="6">
         <v>10</v>
       </c>
-      <c r="B11" s="7"/>
+      <c r="B11" s="6"/>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
-      <c r="H11" s="6"/>
+      <c r="H11" s="7"/>
       <c r="I11" s="7"/>
-      <c r="J11" s="6"/>
-    </row>
-    <row r="12" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J11" s="7"/>
+      <c r="K11" s="6"/>
+    </row>
+    <row r="12" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="6">
         <v>11</v>
       </c>
-      <c r="B12" s="7"/>
+      <c r="B12" s="6"/>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
-      <c r="H12" s="6"/>
+      <c r="H12" s="7"/>
       <c r="I12" s="7"/>
-      <c r="J12" s="6"/>
-    </row>
-    <row r="13" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J12" s="7"/>
+      <c r="K12" s="6"/>
+    </row>
+    <row r="13" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="6">
         <v>12</v>
       </c>
-      <c r="B13" s="7"/>
+      <c r="B13" s="6"/>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
-      <c r="H13" s="6"/>
+      <c r="H13" s="7"/>
       <c r="I13" s="7"/>
-      <c r="J13" s="6"/>
-    </row>
-    <row r="14" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J13" s="7"/>
+      <c r="K13" s="6"/>
+    </row>
+    <row r="14" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="6">
         <v>13</v>
       </c>
-      <c r="B14" s="7"/>
+      <c r="B14" s="6"/>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
       <c r="G14" s="7"/>
-      <c r="H14" s="6"/>
+      <c r="H14" s="7"/>
       <c r="I14" s="7"/>
-      <c r="J14" s="6"/>
-    </row>
-    <row r="15" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J14" s="7"/>
+      <c r="K14" s="6"/>
+    </row>
+    <row r="15" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="6">
         <v>14</v>
       </c>
-      <c r="B15" s="7"/>
+      <c r="B15" s="6"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
       <c r="G15" s="7"/>
-      <c r="H15" s="6"/>
+      <c r="H15" s="7"/>
       <c r="I15" s="7"/>
-      <c r="J15" s="6"/>
-    </row>
-    <row r="16" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J15" s="7"/>
+      <c r="K15" s="6"/>
+    </row>
+    <row r="16" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="6">
         <v>15</v>
       </c>
-      <c r="B16" s="7"/>
+      <c r="B16" s="6"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
       <c r="G16" s="7"/>
-      <c r="H16" s="6"/>
+      <c r="H16" s="7"/>
       <c r="I16" s="7"/>
-      <c r="J16" s="6"/>
-    </row>
-    <row r="17" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J16" s="7"/>
+      <c r="K16" s="6"/>
+    </row>
+    <row r="17" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="6">
         <v>16</v>
       </c>
-      <c r="B17" s="7"/>
+      <c r="B17" s="6"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
       <c r="G17" s="7"/>
-      <c r="H17" s="6"/>
+      <c r="H17" s="7"/>
       <c r="I17" s="7"/>
-      <c r="J17" s="6"/>
-    </row>
-    <row r="18" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J17" s="7"/>
+      <c r="K17" s="6"/>
+    </row>
+    <row r="18" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="6">
         <v>17</v>
       </c>
-      <c r="B18" s="7"/>
+      <c r="B18" s="6"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
-      <c r="H18" s="6"/>
+      <c r="H18" s="7"/>
       <c r="I18" s="7"/>
-      <c r="J18" s="6"/>
-    </row>
-    <row r="19" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J18" s="7"/>
+      <c r="K18" s="6"/>
+    </row>
+    <row r="19" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="6">
         <v>18</v>
       </c>
-      <c r="B19" s="7"/>
+      <c r="B19" s="6"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
-      <c r="H19" s="6"/>
+      <c r="H19" s="7"/>
       <c r="I19" s="7"/>
-      <c r="J19" s="6"/>
-    </row>
-    <row r="20" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J19" s="7"/>
+      <c r="K19" s="6"/>
+    </row>
+    <row r="20" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="6">
         <v>19</v>
       </c>
-      <c r="B20" s="7"/>
+      <c r="B20" s="6"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
       <c r="F20" s="7"/>
       <c r="G20" s="7"/>
-      <c r="H20" s="6"/>
+      <c r="H20" s="7"/>
       <c r="I20" s="7"/>
-      <c r="J20" s="6"/>
-    </row>
-    <row r="21" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J20" s="7"/>
+      <c r="K20" s="6"/>
+    </row>
+    <row r="21" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="6">
         <v>20</v>
       </c>
-      <c r="B21" s="7"/>
+      <c r="B21" s="6"/>
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
       <c r="E21" s="7"/>
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
-      <c r="H21" s="6"/>
+      <c r="H21" s="7"/>
       <c r="I21" s="7"/>
-      <c r="J21" s="6"/>
-    </row>
-    <row r="22" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J21" s="7"/>
+      <c r="K21" s="6"/>
+    </row>
+    <row r="22" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="6">
         <v>21</v>
       </c>
-      <c r="B22" s="7"/>
+      <c r="B22" s="6"/>
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
       <c r="E22" s="7"/>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
-      <c r="H22" s="6"/>
+      <c r="H22" s="7"/>
       <c r="I22" s="7"/>
-      <c r="J22" s="6"/>
-    </row>
-    <row r="23" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J22" s="7"/>
+      <c r="K22" s="6"/>
+    </row>
+    <row r="23" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="6">
         <v>22</v>
       </c>
-      <c r="B23" s="7"/>
+      <c r="B23" s="6"/>
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
       <c r="E23" s="7"/>
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
-      <c r="H23" s="6"/>
+      <c r="H23" s="7"/>
       <c r="I23" s="7"/>
-      <c r="J23" s="6"/>
-    </row>
-    <row r="24" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J23" s="7"/>
+      <c r="K23" s="6"/>
+    </row>
+    <row r="24" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="6">
         <v>23</v>
       </c>
-      <c r="B24" s="7"/>
+      <c r="B24" s="6"/>
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
       <c r="E24" s="7"/>
       <c r="F24" s="7"/>
       <c r="G24" s="7"/>
-      <c r="H24" s="6"/>
+      <c r="H24" s="7"/>
       <c r="I24" s="7"/>
-      <c r="J24" s="6"/>
-    </row>
-    <row r="25" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J24" s="7"/>
+      <c r="K24" s="6"/>
+    </row>
+    <row r="25" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="6">
         <v>24</v>
       </c>
-      <c r="B25" s="7"/>
+      <c r="B25" s="6"/>
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
       <c r="E25" s="7"/>
       <c r="F25" s="7"/>
       <c r="G25" s="7"/>
-      <c r="H25" s="6"/>
+      <c r="H25" s="7"/>
       <c r="I25" s="7"/>
-      <c r="J25" s="6"/>
-    </row>
-    <row r="26" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J25" s="7"/>
+      <c r="K25" s="6"/>
+    </row>
+    <row r="26" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="6">
         <v>25</v>
       </c>
-      <c r="B26" s="7"/>
+      <c r="B26" s="6"/>
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
       <c r="G26" s="7"/>
-      <c r="H26" s="6"/>
+      <c r="H26" s="7"/>
       <c r="I26" s="7"/>
-      <c r="J26" s="6"/>
-    </row>
-    <row r="27" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J26" s="7"/>
+      <c r="K26" s="6"/>
+    </row>
+    <row r="27" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="6">
         <v>26</v>
       </c>
-      <c r="B27" s="7"/>
+      <c r="B27" s="6"/>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
-      <c r="H27" s="6"/>
+      <c r="H27" s="7"/>
       <c r="I27" s="7"/>
-      <c r="J27" s="6"/>
-    </row>
-    <row r="28" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J27" s="7"/>
+      <c r="K27" s="6"/>
+    </row>
+    <row r="28" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="6">
         <v>27</v>
       </c>
-      <c r="B28" s="7"/>
+      <c r="B28" s="6"/>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
       <c r="E28" s="7"/>
       <c r="F28" s="7"/>
       <c r="G28" s="7"/>
-      <c r="H28" s="6"/>
+      <c r="H28" s="7"/>
       <c r="I28" s="7"/>
-      <c r="J28" s="6"/>
-    </row>
-    <row r="29" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J28" s="7"/>
+      <c r="K28" s="6"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="6">
         <v>28</v>
       </c>
-      <c r="B29" s="7"/>
+      <c r="B29" s="6"/>
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
       <c r="E29" s="7"/>
       <c r="F29" s="7"/>
       <c r="G29" s="7"/>
-      <c r="H29" s="6"/>
+      <c r="H29" s="7"/>
       <c r="I29" s="7"/>
-      <c r="J29" s="6"/>
-    </row>
-    <row r="30" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J29" s="7"/>
+      <c r="K29" s="6"/>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="6">
         <v>29</v>
       </c>
-      <c r="B30" s="7"/>
+      <c r="B30" s="6"/>
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
       <c r="E30" s="7"/>
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
-      <c r="H30" s="6"/>
+      <c r="H30" s="7"/>
       <c r="I30" s="7"/>
-      <c r="J30" s="6"/>
-    </row>
-    <row r="31" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J30" s="7"/>
+      <c r="K30" s="6"/>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="6">
         <v>30</v>
       </c>
-      <c r="B31" s="7"/>
+      <c r="B31" s="6"/>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
       <c r="G31" s="7"/>
-      <c r="H31" s="6"/>
+      <c r="H31" s="7"/>
       <c r="I31" s="7"/>
-      <c r="J31" s="6"/>
-    </row>
-    <row r="32" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J31" s="7"/>
+      <c r="K31" s="6"/>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="6">
         <v>31</v>
       </c>
-      <c r="B32" s="7"/>
+      <c r="B32" s="6"/>
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
       <c r="E32" s="7"/>
       <c r="F32" s="7"/>
       <c r="G32" s="7"/>
-      <c r="H32" s="6"/>
+      <c r="H32" s="7"/>
       <c r="I32" s="7"/>
-      <c r="J32" s="6"/>
-    </row>
-    <row r="33" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J32" s="7"/>
+      <c r="K32" s="6"/>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="6">
         <v>32</v>
       </c>
-      <c r="B33" s="7"/>
+      <c r="B33" s="6"/>
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
       <c r="G33" s="7"/>
-      <c r="H33" s="6"/>
+      <c r="H33" s="7"/>
       <c r="I33" s="7"/>
-      <c r="J33" s="6"/>
-    </row>
-    <row r="34" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J33" s="7"/>
+      <c r="K33" s="6"/>
+    </row>
+    <row r="34" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="6">
         <v>33</v>
       </c>
-      <c r="B34" s="7"/>
+      <c r="B34" s="6"/>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
       <c r="E34" s="7"/>
       <c r="F34" s="7"/>
       <c r="G34" s="7"/>
-      <c r="H34" s="6"/>
+      <c r="H34" s="7"/>
       <c r="I34" s="7"/>
-      <c r="J34" s="6"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J34" s="7"/>
+      <c r="K34" s="6"/>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="6">
         <v>34</v>
       </c>
-      <c r="B35" s="7"/>
+      <c r="B35" s="6"/>
       <c r="C35" s="7"/>
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
       <c r="F35" s="7"/>
       <c r="G35" s="7"/>
-      <c r="H35" s="6"/>
+      <c r="H35" s="7"/>
       <c r="I35" s="7"/>
-      <c r="J35" s="6"/>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J35" s="7"/>
+      <c r="K35" s="6"/>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="6">
         <v>35</v>
       </c>
-      <c r="B36" s="7"/>
+      <c r="B36" s="6"/>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
       <c r="F36" s="7"/>
       <c r="G36" s="7"/>
-      <c r="H36" s="6"/>
+      <c r="H36" s="7"/>
       <c r="I36" s="7"/>
-      <c r="J36" s="6"/>
-    </row>
-    <row r="37" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J36" s="7"/>
+      <c r="K36" s="6"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="6">
         <v>36</v>
       </c>
-      <c r="B37" s="7"/>
+      <c r="B37" s="6"/>
       <c r="C37" s="7"/>
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" s="7"/>
       <c r="G37" s="7"/>
-      <c r="H37" s="6"/>
+      <c r="H37" s="7"/>
       <c r="I37" s="7"/>
-      <c r="J37" s="6"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J37" s="7"/>
+      <c r="K37" s="6"/>
+    </row>
+    <row r="38" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="6">
         <v>37</v>
       </c>
-      <c r="B38" s="7"/>
+      <c r="B38" s="6"/>
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
       <c r="F38" s="7"/>
       <c r="G38" s="7"/>
-      <c r="H38" s="6"/>
+      <c r="H38" s="7"/>
       <c r="I38" s="7"/>
-      <c r="J38" s="6"/>
-    </row>
-    <row r="39" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J38" s="7"/>
+      <c r="K38" s="6"/>
+    </row>
+    <row r="39" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="6">
         <v>38</v>
       </c>
-      <c r="B39" s="7"/>
+      <c r="B39" s="6"/>
       <c r="C39" s="7"/>
       <c r="D39" s="7"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
       <c r="G39" s="7"/>
-      <c r="H39" s="6"/>
+      <c r="H39" s="7"/>
       <c r="I39" s="7"/>
-      <c r="J39" s="6"/>
-    </row>
-    <row r="40" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J39" s="7"/>
+      <c r="K39" s="6"/>
+    </row>
+    <row r="40" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="6">
         <v>39</v>
       </c>
-      <c r="B40" s="7"/>
+      <c r="B40" s="6"/>
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
       <c r="E40" s="7"/>
       <c r="F40" s="7"/>
       <c r="G40" s="7"/>
-      <c r="H40" s="6"/>
+      <c r="H40" s="7"/>
       <c r="I40" s="7"/>
-      <c r="J40" s="6"/>
-    </row>
-    <row r="41" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J40" s="7"/>
+      <c r="K40" s="6"/>
+    </row>
+    <row r="41" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="6">
         <v>40</v>
       </c>
-      <c r="B41" s="7"/>
+      <c r="B41" s="6"/>
       <c r="C41" s="7"/>
       <c r="D41" s="7"/>
       <c r="E41" s="7"/>
       <c r="F41" s="7"/>
       <c r="G41" s="7"/>
-      <c r="H41" s="6"/>
+      <c r="H41" s="7"/>
       <c r="I41" s="7"/>
-      <c r="J41" s="6"/>
-    </row>
-    <row r="42" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J41" s="7"/>
+      <c r="K41" s="6"/>
+    </row>
+    <row r="42" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="6">
         <v>41</v>
       </c>
-      <c r="B42" s="7"/>
+      <c r="B42" s="6"/>
       <c r="C42" s="7"/>
       <c r="D42" s="7"/>
       <c r="E42" s="7"/>
       <c r="F42" s="7"/>
       <c r="G42" s="7"/>
-      <c r="H42" s="6"/>
+      <c r="H42" s="7"/>
       <c r="I42" s="7"/>
-      <c r="J42" s="6"/>
-    </row>
-    <row r="43" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J42" s="7"/>
+      <c r="K42" s="6"/>
+    </row>
+    <row r="43" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="6">
         <v>42</v>
       </c>
-      <c r="B43" s="7"/>
+      <c r="B43" s="6"/>
       <c r="C43" s="7"/>
       <c r="D43" s="7"/>
       <c r="E43" s="7"/>
       <c r="F43" s="7"/>
       <c r="G43" s="7"/>
-      <c r="H43" s="6"/>
+      <c r="H43" s="7"/>
       <c r="I43" s="7"/>
-      <c r="J43" s="6"/>
-    </row>
-    <row r="44" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J43" s="7"/>
+      <c r="K43" s="6"/>
+    </row>
+    <row r="44" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="6">
         <v>43</v>
       </c>
-      <c r="B44" s="7"/>
+      <c r="B44" s="6"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
       <c r="G44" s="7"/>
-      <c r="H44" s="6"/>
+      <c r="H44" s="7"/>
       <c r="I44" s="7"/>
-      <c r="J44" s="6"/>
-    </row>
-    <row r="45" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J44" s="7"/>
+      <c r="K44" s="6"/>
+    </row>
+    <row r="45" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="6">
         <v>44</v>
       </c>
-      <c r="B45" s="7"/>
+      <c r="B45" s="6"/>
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
       <c r="E45" s="7"/>
       <c r="F45" s="7"/>
       <c r="G45" s="7"/>
-      <c r="H45" s="6"/>
+      <c r="H45" s="7"/>
       <c r="I45" s="7"/>
-      <c r="J45" s="6"/>
-    </row>
-    <row r="46" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J45" s="7"/>
+      <c r="K45" s="6"/>
+    </row>
+    <row r="46" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="6">
         <v>45</v>
       </c>
-      <c r="B46" s="7"/>
+      <c r="B46" s="6"/>
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
       <c r="F46" s="7"/>
       <c r="G46" s="7"/>
-      <c r="H46" s="6"/>
+      <c r="H46" s="7"/>
       <c r="I46" s="7"/>
-      <c r="J46" s="6"/>
-    </row>
-    <row r="47" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J46" s="7"/>
+      <c r="K46" s="6"/>
+    </row>
+    <row r="47" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="6">
         <v>46</v>
       </c>
-      <c r="B47" s="7"/>
+      <c r="B47" s="6"/>
       <c r="C47" s="7"/>
       <c r="D47" s="7"/>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
       <c r="G47" s="7"/>
-      <c r="H47" s="6"/>
+      <c r="H47" s="7"/>
       <c r="I47" s="7"/>
-      <c r="J47" s="6"/>
-    </row>
-    <row r="48" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J47" s="7"/>
+      <c r="K47" s="6"/>
+    </row>
+    <row r="48" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="6">
         <v>47</v>
       </c>
-      <c r="B48" s="7"/>
+      <c r="B48" s="6"/>
       <c r="C48" s="7"/>
       <c r="D48" s="7"/>
       <c r="E48" s="7"/>
       <c r="F48" s="7"/>
       <c r="G48" s="7"/>
-      <c r="H48" s="6"/>
+      <c r="H48" s="7"/>
       <c r="I48" s="7"/>
-      <c r="J48" s="6"/>
-    </row>
-    <row r="49" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J48" s="7"/>
+      <c r="K48" s="6"/>
+    </row>
+    <row r="49" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="6">
         <v>48</v>
       </c>
-      <c r="B49" s="7"/>
+      <c r="B49" s="6"/>
       <c r="C49" s="7"/>
       <c r="D49" s="7"/>
       <c r="E49" s="7"/>
       <c r="F49" s="7"/>
       <c r="G49" s="7"/>
-      <c r="H49" s="6"/>
+      <c r="H49" s="7"/>
       <c r="I49" s="7"/>
-      <c r="J49" s="6"/>
-    </row>
-    <row r="50" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J49" s="7"/>
+      <c r="K49" s="6"/>
+    </row>
+    <row r="50" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="6">
         <v>49</v>
       </c>
-      <c r="B50" s="7"/>
+      <c r="B50" s="6"/>
       <c r="C50" s="7"/>
       <c r="D50" s="7"/>
       <c r="E50" s="7"/>
       <c r="F50" s="7"/>
       <c r="G50" s="7"/>
-      <c r="H50" s="6"/>
+      <c r="H50" s="7"/>
       <c r="I50" s="7"/>
-      <c r="J50" s="6"/>
-    </row>
-    <row r="51" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J50" s="7"/>
+      <c r="K50" s="6"/>
+    </row>
+    <row r="51" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="6">
         <v>50</v>
       </c>
-      <c r="B51" s="7"/>
+      <c r="B51" s="6"/>
       <c r="C51" s="7"/>
       <c r="D51" s="7"/>
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
       <c r="G51" s="7"/>
-      <c r="H51" s="6"/>
+      <c r="H51" s="7"/>
       <c r="I51" s="7"/>
-      <c r="J51" s="6"/>
-    </row>
-    <row r="52" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J51" s="7"/>
+      <c r="K51" s="6"/>
+    </row>
+    <row r="52" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="6">
         <v>51</v>
       </c>
-      <c r="B52" s="7"/>
+      <c r="B52" s="6"/>
       <c r="C52" s="7"/>
       <c r="D52" s="7"/>
       <c r="E52" s="7"/>
       <c r="F52" s="7"/>
       <c r="G52" s="7"/>
-      <c r="H52" s="6"/>
+      <c r="H52" s="7"/>
       <c r="I52" s="7"/>
-      <c r="J52" s="6"/>
-    </row>
-    <row r="53" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J52" s="7"/>
+      <c r="K52" s="6"/>
+    </row>
+    <row r="53" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="6">
         <v>52</v>
       </c>
-      <c r="B53" s="7"/>
+      <c r="B53" s="6"/>
       <c r="C53" s="7"/>
       <c r="D53" s="7"/>
       <c r="E53" s="7"/>
       <c r="F53" s="7"/>
       <c r="G53" s="7"/>
-      <c r="H53" s="6"/>
+      <c r="H53" s="7"/>
       <c r="I53" s="7"/>
-      <c r="J53" s="6"/>
-    </row>
-    <row r="54" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J53" s="7"/>
+      <c r="K53" s="6"/>
+    </row>
+    <row r="54" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="6">
         <v>53</v>
       </c>
-      <c r="B54" s="7"/>
+      <c r="B54" s="6"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
       <c r="E54" s="7"/>
       <c r="F54" s="7"/>
       <c r="G54" s="7"/>
-      <c r="H54" s="6"/>
+      <c r="H54" s="7"/>
       <c r="I54" s="7"/>
-      <c r="J54" s="6"/>
-    </row>
-    <row r="55" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J54" s="7"/>
+      <c r="K54" s="6"/>
+    </row>
+    <row r="55" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="6">
         <v>54</v>
       </c>
-      <c r="B55" s="7"/>
+      <c r="B55" s="6"/>
       <c r="C55" s="7"/>
       <c r="D55" s="7"/>
       <c r="E55" s="7"/>
       <c r="F55" s="7"/>
       <c r="G55" s="7"/>
-      <c r="H55" s="6"/>
+      <c r="H55" s="7"/>
       <c r="I55" s="7"/>
-      <c r="J55" s="6"/>
-    </row>
-    <row r="56" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J55" s="7"/>
+      <c r="K55" s="6"/>
+    </row>
+    <row r="56" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="6">
         <v>55</v>
       </c>
-      <c r="B56" s="7"/>
+      <c r="B56" s="6"/>
       <c r="C56" s="7"/>
       <c r="D56" s="7"/>
       <c r="E56" s="7"/>
       <c r="F56" s="7"/>
       <c r="G56" s="7"/>
-      <c r="H56" s="6"/>
+      <c r="H56" s="7"/>
       <c r="I56" s="7"/>
-      <c r="J56" s="6"/>
-    </row>
-    <row r="57" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J56" s="7"/>
+      <c r="K56" s="6"/>
+    </row>
+    <row r="57" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="6">
         <v>56</v>
       </c>
-      <c r="B57" s="7"/>
+      <c r="B57" s="6"/>
       <c r="C57" s="7"/>
       <c r="D57" s="7"/>
       <c r="E57" s="7"/>
       <c r="F57" s="7"/>
       <c r="G57" s="7"/>
-      <c r="H57" s="6"/>
+      <c r="H57" s="7"/>
       <c r="I57" s="7"/>
-      <c r="J57" s="6"/>
-    </row>
-    <row r="58" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J57" s="7"/>
+      <c r="K57" s="6"/>
+    </row>
+    <row r="58" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="6">
         <v>57</v>
       </c>
-      <c r="B58" s="7"/>
+      <c r="B58" s="6"/>
       <c r="C58" s="7"/>
       <c r="D58" s="7"/>
       <c r="E58" s="7"/>
       <c r="F58" s="7"/>
       <c r="G58" s="7"/>
-      <c r="H58" s="6"/>
+      <c r="H58" s="7"/>
       <c r="I58" s="7"/>
-      <c r="J58" s="6"/>
-    </row>
-    <row r="59" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J58" s="7"/>
+      <c r="K58" s="6"/>
+    </row>
+    <row r="59" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="6">
         <v>58</v>
       </c>
-      <c r="B59" s="7"/>
+      <c r="B59" s="6"/>
       <c r="C59" s="7"/>
       <c r="D59" s="7"/>
       <c r="E59" s="7"/>
       <c r="F59" s="7"/>
       <c r="G59" s="7"/>
-      <c r="H59" s="6"/>
+      <c r="H59" s="7"/>
       <c r="I59" s="7"/>
-      <c r="J59" s="6"/>
-    </row>
-    <row r="60" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J59" s="7"/>
+      <c r="K59" s="6"/>
+    </row>
+    <row r="60" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="6">
         <v>59</v>
       </c>
-      <c r="B60" s="7"/>
+      <c r="B60" s="6"/>
       <c r="C60" s="7"/>
       <c r="D60" s="7"/>
       <c r="E60" s="7"/>
       <c r="F60" s="7"/>
       <c r="G60" s="7"/>
-      <c r="H60" s="6"/>
+      <c r="H60" s="7"/>
       <c r="I60" s="7"/>
-      <c r="J60" s="6"/>
+      <c r="J60" s="7"/>
+      <c r="K60" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Pilihan Tidak Valid" error="Kunci jawaban harus berupa salah satu huruf: A, B, C, D, atau E" sqref="H10:H60">
-      <formula1>"A,B,C,D,E"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Tipe Soal Tidak Valid" error="Pilihlah salah satu tipe soal yang tersedia dari menu dropdown" sqref="B10:B60">
+      <formula1>"PILIHAN GANDA,PG KOMPLEKS,BENAR SALAH,ISIAN SINGKAT,MENJODOHKAN,ESAI"</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Pilihan Tidak Valid" error="Kunci jawaban harus berupa salah satu huruf: A, B, C, D, atau E" sqref="H2:H60">
-      <formula1>"A,B,C,D,E"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Tipe Soal Tidak Valid" error="Pilihlah salah satu tipe soal yang tersedia dari menu dropdown" sqref="B2:B60">
+      <formula1>"PILIHAN GANDA,PG KOMPLEKS,BENAR SALAH,ISIAN SINGKAT,MENJODOHKAN,ESAI"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Kesulitan Tidak Valid" error="Tingkat kesulitan harus berupa: MUDAH, SEDANG, atau SULIT" sqref="J10:J60">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Kesulitan Tidak Valid" error="Tingkat kesulitan harus berupa: MUDAH, SEDANG, atau SULIT" sqref="K10:K60">
       <formula1>"MUDAH,SEDANG,SULIT"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Kesulitan Tidak Valid" error="Tingkat kesulitan harus berupa: MUDAH, SEDANG, atau SULIT" sqref="J2:J60">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Kesulitan Tidak Valid" error="Tingkat kesulitan harus berupa: MUDAH, SEDANG, atau SULIT" sqref="K2:K60">
       <formula1>"MUDAH,SEDANG,SULIT"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="F59E0B"/>
-  </sheetPr>
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="3" max="7" width="25" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="35" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="6">
-        <v>1</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="6">
-        <v>2</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="6">
-        <v>3</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
 </file>
</xml_diff>